<commit_message>
More notes on ker3
Added some more documentation and notes on kern3
</commit_message>
<xml_diff>
--- a/cuda_optimize/graphs/sgemm_performance_graphs.xlsx
+++ b/cuda_optimize/graphs/sgemm_performance_graphs.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\conor\source\repos\texashodlr\coding-and-curling\cuda_optimize\graphs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B37F76EE-C2F8-4BDA-AB1B-7E97AAA7D48E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E68F0FBD-4AB9-4FBB-8FEE-1A714569859A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-19290" yWindow="-10670" windowWidth="19380" windowHeight="20970" activeTab="1" xr2:uid="{603C1C53-CEB8-463D-A515-B200F43602F4}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="2" activeTab="2" xr2:uid="{603C1C53-CEB8-463D-A515-B200F43602F4}"/>
   </bookViews>
   <sheets>
     <sheet name="kernel_1_naive" sheetId="1" r:id="rId1"/>
     <sheet name="kernel_2_gmem_coal" sheetId="2" r:id="rId2"/>
+    <sheet name="kernel_3_shmem_cache" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="3">
   <si>
     <t>Dimensions (M=N=K)</t>
   </si>
@@ -1248,6 +1249,664 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000000-5251-48BD-9AD5-8586FDBC7B1E}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="765405536"/>
+        <c:axId val="765411776"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="765405536"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="765411776"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="765411776"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="765405536"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>kernel_3_shmem_cache!$D$4</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Performance (GFLOPS)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>kernel_3_shmem_cache!$B$5:$B$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>128</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>256</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>512</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1024</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2048</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>4096</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>kernel_3_shmem_cache!$D$5:$D$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>254.7</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1084.4000000000001</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1276.5999999999999</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1435.9</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1776.1</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1632.5</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-E3ED-45E0-9B79-E0C9E83C5AC3}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="765441056"/>
+        <c:axId val="765437696"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="765441056"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="765437696"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="765437696"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="765441056"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>kernel_3_shmem_cache!$C$4</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Avg. Elapsed Time (s)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>kernel_3_shmem_cache!$B$5:$B$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>128</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>256</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>512</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1024</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2048</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>4096</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>kernel_3_shmem_cache!$C$5:$C$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>1.5999999999999999E-5</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3.1000000000000001E-5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2.1000000000000001E-4</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1.4959999999999999E-3</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>9.6729999999999993E-3</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>8.4190000000000001E-2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-E987-4D2E-9796-9A6D12C3F4C5}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1591,6 +2250,86 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors5.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors6.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
@@ -3140,6 +3879,1038 @@
 </file>
 
 <file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style5.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style6.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -3791,6 +5562,87 @@
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{37414488-5FDF-45D3-AB57-FF186BE504A0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>352425</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>47625</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E371F9F5-0D2E-4385-B9E4-CCDB6AEBB84C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>15512</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>318498</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>159839</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1B796AED-3F5F-431C-9C2A-38990CB4DA3E}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -4290,7 +6142,7 @@
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B8">
-        <f t="shared" ref="B8:B11" si="0">2*B7</f>
+        <f t="shared" ref="B8:B10" si="0">2*B7</f>
         <v>1024</v>
       </c>
       <c r="C8">
@@ -4322,6 +6174,101 @@
       </c>
       <c r="D10">
         <v>1062.9000000000001</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A1D697F-FE79-4179-84C2-7892A8237BF1}">
+  <dimension ref="B4:D10"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="10.5546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B4" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B5">
+        <v>128</v>
+      </c>
+      <c r="C5">
+        <v>1.5999999999999999E-5</v>
+      </c>
+      <c r="D5">
+        <v>254.7</v>
+      </c>
+    </row>
+    <row r="6" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B6">
+        <v>256</v>
+      </c>
+      <c r="C6">
+        <v>3.1000000000000001E-5</v>
+      </c>
+      <c r="D6">
+        <v>1084.4000000000001</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B7">
+        <f>2*B6</f>
+        <v>512</v>
+      </c>
+      <c r="C7">
+        <v>2.1000000000000001E-4</v>
+      </c>
+      <c r="D7">
+        <v>1276.5999999999999</v>
+      </c>
+    </row>
+    <row r="8" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B8">
+        <f t="shared" ref="B8:B10" si="0">2*B7</f>
+        <v>1024</v>
+      </c>
+      <c r="C8">
+        <v>1.4959999999999999E-3</v>
+      </c>
+      <c r="D8">
+        <v>1435.9</v>
+      </c>
+    </row>
+    <row r="9" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B9">
+        <f t="shared" si="0"/>
+        <v>2048</v>
+      </c>
+      <c r="C9">
+        <v>9.6729999999999993E-3</v>
+      </c>
+      <c r="D9">
+        <v>1776.1</v>
+      </c>
+    </row>
+    <row r="10" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B10">
+        <f t="shared" si="0"/>
+        <v>4096</v>
+      </c>
+      <c r="C10">
+        <v>8.4190000000000001E-2</v>
+      </c>
+      <c r="D10">
+        <v>1632.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Kernel 5 2D Block tiling
</commit_message>
<xml_diff>
--- a/cuda_optimize/graphs/sgemm_performance_graphs.xlsx
+++ b/cuda_optimize/graphs/sgemm_performance_graphs.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\conor\source\repos\texashodlr\coding-and-curling\cuda_optimize\graphs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{669501E4-ED05-40BA-8BF6-27F3A81DDB6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A349806-C4CC-443A-A968-A1617B4A0761}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="384" yWindow="384" windowWidth="17280" windowHeight="8880" firstSheet="2" activeTab="2" xr2:uid="{603C1C53-CEB8-463D-A515-B200F43602F4}"/>
+    <workbookView xWindow="10572" yWindow="156" windowWidth="17280" windowHeight="8880" firstSheet="2" activeTab="4" xr2:uid="{603C1C53-CEB8-463D-A515-B200F43602F4}"/>
   </bookViews>
   <sheets>
     <sheet name="kernel_1_naive" sheetId="1" r:id="rId1"/>
     <sheet name="kernel_2_gmem_coal" sheetId="2" r:id="rId2"/>
-    <sheet name="kernel_4_gmem_1D" sheetId="4" r:id="rId3"/>
-    <sheet name="kernel_3_shmem_cache" sheetId="3" r:id="rId4"/>
+    <sheet name="kernel_3_shmem_cache" sheetId="3" r:id="rId3"/>
+    <sheet name="kernel_4_gmem_1D" sheetId="4" r:id="rId4"/>
+    <sheet name="kernel_5_shmem_2d" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="3">
   <si>
     <t>Dimensions (M=N=K)</t>
   </si>
@@ -392,6 +393,335 @@
           </a:p>
         </c:txPr>
         <c:crossAx val="765441056"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart10.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>kernel_5_shmem_2d!$C$4</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Avg. Elapsed Time (s)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>kernel_5_shmem_2d!$B$5:$B$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>128</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>256</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>512</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1024</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2048</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>4096</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>kernel_5_shmem_2d!$C$5:$C$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>3.6000000000000001E-5</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>5.3000000000000001E-5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>9.6000000000000002E-5</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3.1700000000000001E-4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2.4580000000000001E-3</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2.2058000000000001E-2</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-00E1-4DEE-AFE8-6C6B2DDEE0B6}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="765405536"/>
+        <c:axId val="765411776"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="765405536"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="765411776"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="765411776"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="765405536"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -1488,7 +1818,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>kernel_4_gmem_1D!$D$4</c:f>
+              <c:f>kernel_3_shmem_cache!$D$4</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1523,7 +1853,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>kernel_4_gmem_1D!$B$5:$B$11</c:f>
+              <c:f>kernel_3_shmem_cache!$B$5:$B$11</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="7"/>
@@ -1550,27 +1880,27 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>kernel_4_gmem_1D!$D$5:$D$11</c:f>
+              <c:f>kernel_3_shmem_cache!$D$5:$D$11</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="7"/>
                 <c:pt idx="0">
-                  <c:v>245.2</c:v>
+                  <c:v>254.7</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1299.2</c:v>
+                  <c:v>1084.4000000000001</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>3574.3</c:v>
+                  <c:v>1276.5999999999999</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>4017.2</c:v>
+                  <c:v>1435.9</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>4592.2</c:v>
+                  <c:v>1776.1</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>4469.2</c:v>
+                  <c:v>1632.5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1578,7 +1908,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-AC30-4F85-BD1A-F9D99BE79747}"/>
+              <c16:uniqueId val="{00000000-E3ED-45E0-9B79-E0C9E83C5AC3}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1817,7 +2147,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>kernel_4_gmem_1D!$C$4</c:f>
+              <c:f>kernel_3_shmem_cache!$C$4</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1852,7 +2182,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>kernel_4_gmem_1D!$B$5:$B$11</c:f>
+              <c:f>kernel_3_shmem_cache!$B$5:$B$11</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="7"/>
@@ -1879,27 +2209,27 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>kernel_4_gmem_1D!$C$5:$C$11</c:f>
+              <c:f>kernel_3_shmem_cache!$C$5:$C$11</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="7"/>
                 <c:pt idx="0">
-                  <c:v>1.7E-5</c:v>
+                  <c:v>1.5999999999999999E-5</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2.5999999999999998E-5</c:v>
+                  <c:v>3.1000000000000001E-5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>7.4999999999999993E-5</c:v>
+                  <c:v>2.1000000000000001E-4</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5.3499999999999999E-4</c:v>
+                  <c:v>1.4959999999999999E-3</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>3.741E-3</c:v>
+                  <c:v>9.6729999999999993E-3</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>3.0752000000000002E-2</c:v>
+                  <c:v>8.4190000000000001E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1907,7 +2237,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-4DA1-465D-86C7-6E993881E6E8}"/>
+              <c16:uniqueId val="{00000000-E987-4D2E-9796-9A6D12C3F4C5}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2146,7 +2476,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>kernel_3_shmem_cache!$D$4</c:f>
+              <c:f>kernel_4_gmem_1D!$D$4</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -2181,7 +2511,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>kernel_3_shmem_cache!$B$5:$B$11</c:f>
+              <c:f>kernel_4_gmem_1D!$B$5:$B$11</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="7"/>
@@ -2208,27 +2538,27 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>kernel_3_shmem_cache!$D$5:$D$11</c:f>
+              <c:f>kernel_4_gmem_1D!$D$5:$D$11</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="7"/>
                 <c:pt idx="0">
-                  <c:v>254.7</c:v>
+                  <c:v>245.2</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1084.4000000000001</c:v>
+                  <c:v>1299.2</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1276.5999999999999</c:v>
+                  <c:v>3574.3</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1435.9</c:v>
+                  <c:v>4017.2</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1776.1</c:v>
+                  <c:v>4592.2</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1632.5</c:v>
+                  <c:v>4469.2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2236,7 +2566,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-E3ED-45E0-9B79-E0C9E83C5AC3}"/>
+              <c16:uniqueId val="{00000000-AC30-4F85-BD1A-F9D99BE79747}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2475,7 +2805,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>kernel_3_shmem_cache!$C$4</c:f>
+              <c:f>kernel_4_gmem_1D!$C$4</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -2510,7 +2840,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>kernel_3_shmem_cache!$B$5:$B$11</c:f>
+              <c:f>kernel_4_gmem_1D!$B$5:$B$11</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="7"/>
@@ -2537,27 +2867,27 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>kernel_3_shmem_cache!$C$5:$C$11</c:f>
+              <c:f>kernel_4_gmem_1D!$C$5:$C$11</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="7"/>
                 <c:pt idx="0">
-                  <c:v>1.5999999999999999E-5</c:v>
+                  <c:v>1.7E-5</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3.1000000000000001E-5</c:v>
+                  <c:v>2.5999999999999998E-5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2.1000000000000001E-4</c:v>
+                  <c:v>7.4999999999999993E-5</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1.4959999999999999E-3</c:v>
+                  <c:v>5.3499999999999999E-4</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>9.6729999999999993E-3</c:v>
+                  <c:v>3.741E-3</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>8.4190000000000001E-2</c:v>
+                  <c:v>3.0752000000000002E-2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2565,7 +2895,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-E987-4D2E-9796-9A6D12C3F4C5}"/>
+              <c16:uniqueId val="{00000000-4DA1-465D-86C7-6E993881E6E8}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2749,7 +3079,376 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart9.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>kernel_5_shmem_2d!$D$4</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Performance (GFLOPS)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>kernel_5_shmem_2d!$B$5:$B$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>128</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>256</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>512</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1024</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2048</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>4096</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>kernel_5_shmem_2d!$D$5:$D$11</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>117.8</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>629.70000000000005</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2803.9</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>6785</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>6988.3</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6230.9</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-A9AB-4C0D-8DB5-A3DF4C7862D7}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="765441056"/>
+        <c:axId val="765437696"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="765441056"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="765437696"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="765437696"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="765441056"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors10.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -3069,6 +3768,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors9.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
@@ -3585,7 +4324,7 @@
 </cs:chartStyle>
 </file>
 
-<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/style10.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -4101,7 +4840,7 @@
 </cs:chartStyle>
 </file>
 
-<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -4617,7 +5356,7 @@
 </cs:chartStyle>
 </file>
 
-<file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -5133,7 +5872,7 @@
 </cs:chartStyle>
 </file>
 
-<file path=xl/charts/style5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -5649,7 +6388,7 @@
 </cs:chartStyle>
 </file>
 
-<file path=xl/charts/style6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/style5.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -6165,7 +6904,7 @@
 </cs:chartStyle>
 </file>
 
-<file path=xl/charts/style7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/style6.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -6681,7 +7420,1039 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style7.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/charts/style8.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style9.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -7375,6 +9146,87 @@
         <xdr:cNvPr id="2" name="Chart 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E371F9F5-0D2E-4385-B9E4-CCDB6AEBB84C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>15512</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>318498</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>159839</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1B796AED-3F5F-431C-9C2A-38990CB4DA3E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>352425</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>47625</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C8491EC9-2505-4C34-9E0E-AEC0209C9742}"/>
             </a:ext>
           </a:extLst>
@@ -7436,7 +9288,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
@@ -7456,7 +9308,7 @@
         <xdr:cNvPr id="2" name="Chart 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E371F9F5-0D2E-4385-B9E4-CCDB6AEBB84C}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D7328310-CF06-47BA-B93F-943759D0850C}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -7494,7 +9346,7 @@
         <xdr:cNvPr id="3" name="Chart 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1B796AED-3F5F-431C-9C2A-38990CB4DA3E}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5CD32FB9-396F-425C-8705-A42687A502EA}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -8035,6 +9887,101 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A1D697F-FE79-4179-84C2-7892A8237BF1}">
+  <dimension ref="B4:D10"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="10.5546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B4" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B5">
+        <v>128</v>
+      </c>
+      <c r="C5">
+        <v>1.5999999999999999E-5</v>
+      </c>
+      <c r="D5">
+        <v>254.7</v>
+      </c>
+    </row>
+    <row r="6" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B6">
+        <v>256</v>
+      </c>
+      <c r="C6">
+        <v>3.1000000000000001E-5</v>
+      </c>
+      <c r="D6">
+        <v>1084.4000000000001</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B7">
+        <f>2*B6</f>
+        <v>512</v>
+      </c>
+      <c r="C7">
+        <v>2.1000000000000001E-4</v>
+      </c>
+      <c r="D7">
+        <v>1276.5999999999999</v>
+      </c>
+    </row>
+    <row r="8" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B8">
+        <f t="shared" ref="B8:B10" si="0">2*B7</f>
+        <v>1024</v>
+      </c>
+      <c r="C8">
+        <v>1.4959999999999999E-3</v>
+      </c>
+      <c r="D8">
+        <v>1435.9</v>
+      </c>
+    </row>
+    <row r="9" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B9">
+        <f t="shared" si="0"/>
+        <v>2048</v>
+      </c>
+      <c r="C9">
+        <v>9.6729999999999993E-3</v>
+      </c>
+      <c r="D9">
+        <v>1776.1</v>
+      </c>
+    </row>
+    <row r="10" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B10">
+        <f t="shared" si="0"/>
+        <v>4096</v>
+      </c>
+      <c r="C10">
+        <v>8.4190000000000001E-2</v>
+      </c>
+      <c r="D10">
+        <v>1632.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E304EEC9-1F88-4EC6-80C8-2E0EFD879725}">
   <dimension ref="B4:D10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -8129,8 +10076,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A1D697F-FE79-4179-84C2-7892A8237BF1}">
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{72A8A70A-2389-491B-818A-C3A3D749CED1}">
   <dimension ref="B4:D10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -8153,10 +10100,10 @@
         <v>128</v>
       </c>
       <c r="C5">
-        <v>1.5999999999999999E-5</v>
+        <v>3.6000000000000001E-5</v>
       </c>
       <c r="D5">
-        <v>254.7</v>
+        <v>117.8</v>
       </c>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.3">
@@ -8164,10 +10111,10 @@
         <v>256</v>
       </c>
       <c r="C6">
-        <v>3.1000000000000001E-5</v>
+        <v>5.3000000000000001E-5</v>
       </c>
       <c r="D6">
-        <v>1084.4000000000001</v>
+        <v>629.70000000000005</v>
       </c>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.3">
@@ -8176,10 +10123,10 @@
         <v>512</v>
       </c>
       <c r="C7">
-        <v>2.1000000000000001E-4</v>
+        <v>9.6000000000000002E-5</v>
       </c>
       <c r="D7">
-        <v>1276.5999999999999</v>
+        <v>2803.9</v>
       </c>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.3">
@@ -8188,10 +10135,10 @@
         <v>1024</v>
       </c>
       <c r="C8">
-        <v>1.4959999999999999E-3</v>
+        <v>3.1700000000000001E-4</v>
       </c>
       <c r="D8">
-        <v>1435.9</v>
+        <v>6785</v>
       </c>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.3">
@@ -8200,10 +10147,10 @@
         <v>2048</v>
       </c>
       <c r="C9">
-        <v>9.6729999999999993E-3</v>
+        <v>2.4580000000000001E-3</v>
       </c>
       <c r="D9">
-        <v>1776.1</v>
+        <v>6988.3</v>
       </c>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.3">
@@ -8212,10 +10159,10 @@
         <v>4096</v>
       </c>
       <c r="C10">
-        <v>8.4190000000000001E-2</v>
+        <v>2.2058000000000001E-2</v>
       </c>
       <c r="D10">
-        <v>1632.5</v>
+        <v>6230.9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>